<commit_message>
fix: table_writer(인정, 종합) 수정 및 demo_validator 에 임 시공휴일 예외처리
인정조사, 종합조사에 대한 단가표 작성 시 상대 위치 기반->키워드(1구간, 1등급 등) 기반으로 탐색하도록 코드 수정

20
25년 결제단가표 생성 후 원활한 검증을 위해 임시공휴일 관련 행은 검증 대상에서 제외

해당 코드에 대해 2025, 2026년도 기본, 추가, 결제 단 가표가 완벽하게 생성되는 것을 확인하였음
</commit_message>
<xml_diff>
--- a/xlsx_files/추가급여_단가표.xlsx
+++ b/xlsx_files/추가급여_단가표.xlsx
@@ -473,10 +473,10 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E2" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -507,10 +507,10 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E3" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -541,13 +541,13 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E4" t="n">
-        <v>1357300</v>
+        <v>1305400</v>
       </c>
       <c r="F4" t="n">
-        <v>27700</v>
+        <v>26600</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -575,13 +575,13 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E5" t="n">
-        <v>1343500</v>
+        <v>1292100</v>
       </c>
       <c r="F5" t="n">
-        <v>41500</v>
+        <v>39900</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -609,13 +609,13 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E6" t="n">
-        <v>1329600</v>
+        <v>1278800</v>
       </c>
       <c r="F6" t="n">
-        <v>55400</v>
+        <v>53200</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -643,13 +643,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E7" t="n">
-        <v>1315800</v>
+        <v>1265400</v>
       </c>
       <c r="F7" t="n">
-        <v>69200</v>
+        <v>66600</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -677,10 +677,10 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="E8" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -711,10 +711,10 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="E9" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -745,13 +745,13 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="E10" t="n">
-        <v>171500</v>
+        <v>164700</v>
       </c>
       <c r="F10" t="n">
-        <v>3500</v>
+        <v>3300</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -779,13 +779,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="E11" t="n">
-        <v>169800</v>
+        <v>163000</v>
       </c>
       <c r="F11" t="n">
-        <v>5200</v>
+        <v>5000</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -813,13 +813,13 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="E12" t="n">
-        <v>168000</v>
+        <v>161300</v>
       </c>
       <c r="F12" t="n">
-        <v>7000</v>
+        <v>6700</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -847,13 +847,13 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>175000</v>
+        <v>168000</v>
       </c>
       <c r="E13" t="n">
-        <v>166300</v>
+        <v>159600</v>
       </c>
       <c r="F13" t="n">
-        <v>8700</v>
+        <v>8400</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -881,10 +881,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="E14" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -915,10 +915,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="E15" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -949,13 +949,13 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="E16" t="n">
-        <v>680200</v>
+        <v>653700</v>
       </c>
       <c r="F16" t="n">
-        <v>13800</v>
+        <v>13300</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -983,13 +983,13 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="E17" t="n">
-        <v>673200</v>
+        <v>647000</v>
       </c>
       <c r="F17" t="n">
-        <v>20800</v>
+        <v>20000</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1017,13 +1017,13 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="E18" t="n">
-        <v>666300</v>
+        <v>640400</v>
       </c>
       <c r="F18" t="n">
-        <v>27700</v>
+        <v>26600</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1051,13 +1051,13 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>694000</v>
+        <v>667000</v>
       </c>
       <c r="E19" t="n">
-        <v>659300</v>
+        <v>633700</v>
       </c>
       <c r="F19" t="n">
-        <v>34700</v>
+        <v>33300</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1085,10 +1085,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E20" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1119,10 +1119,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E21" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1153,13 +1153,13 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E22" t="n">
-        <v>342100</v>
+        <v>328300</v>
       </c>
       <c r="F22" t="n">
-        <v>6900</v>
+        <v>6700</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -1187,13 +1187,13 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E23" t="n">
-        <v>338600</v>
+        <v>325000</v>
       </c>
       <c r="F23" t="n">
-        <v>10400</v>
+        <v>10000</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -1221,13 +1221,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E24" t="n">
-        <v>335100</v>
+        <v>321600</v>
       </c>
       <c r="F24" t="n">
-        <v>13900</v>
+        <v>13400</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -1255,13 +1255,13 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E25" t="n">
-        <v>331600</v>
+        <v>318300</v>
       </c>
       <c r="F25" t="n">
-        <v>17400</v>
+        <v>16700</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -1289,10 +1289,10 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E26" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1323,10 +1323,10 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E27" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1357,13 +1357,13 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E28" t="n">
-        <v>342100</v>
+        <v>328300</v>
       </c>
       <c r="F28" t="n">
-        <v>6900</v>
+        <v>6700</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1391,13 +1391,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E29" t="n">
-        <v>338600</v>
+        <v>325000</v>
       </c>
       <c r="F29" t="n">
-        <v>10400</v>
+        <v>10000</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -1425,13 +1425,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E30" t="n">
-        <v>335100</v>
+        <v>321600</v>
       </c>
       <c r="F30" t="n">
-        <v>13900</v>
+        <v>13400</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1459,13 +1459,13 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E31" t="n">
-        <v>331600</v>
+        <v>318300</v>
       </c>
       <c r="F31" t="n">
-        <v>17400</v>
+        <v>16700</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1493,10 +1493,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="E32" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1527,10 +1527,10 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="E33" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1561,13 +1561,13 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="E34" t="n">
-        <v>1238800</v>
+        <v>1191700</v>
       </c>
       <c r="F34" t="n">
-        <v>25200</v>
+        <v>24300</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1595,13 +1595,13 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="E35" t="n">
-        <v>1226100</v>
+        <v>1179600</v>
       </c>
       <c r="F35" t="n">
-        <v>37900</v>
+        <v>36400</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -1629,13 +1629,13 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="E36" t="n">
-        <v>1213500</v>
+        <v>1167400</v>
       </c>
       <c r="F36" t="n">
-        <v>50500</v>
+        <v>48600</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -1663,13 +1663,13 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1264000</v>
+        <v>1216000</v>
       </c>
       <c r="E37" t="n">
-        <v>1200800</v>
+        <v>1155200</v>
       </c>
       <c r="F37" t="n">
-        <v>63200</v>
+        <v>60800</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -1697,10 +1697,10 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E38" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -1731,10 +1731,10 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E39" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -1765,13 +1765,13 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E40" t="n">
-        <v>4623700</v>
+        <v>4449200</v>
       </c>
       <c r="F40" t="n">
-        <v>94300</v>
+        <v>90800</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -1799,13 +1799,13 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E41" t="n">
-        <v>4576500</v>
+        <v>4403800</v>
       </c>
       <c r="F41" t="n">
-        <v>141500</v>
+        <v>136200</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -1833,13 +1833,13 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E42" t="n">
-        <v>4529300</v>
+        <v>4358400</v>
       </c>
       <c r="F42" t="n">
-        <v>188700</v>
+        <v>181600</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -1867,13 +1867,13 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E43" t="n">
-        <v>4482100</v>
+        <v>4313000</v>
       </c>
       <c r="F43" t="n">
-        <v>235900</v>
+        <v>227000</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -1901,10 +1901,10 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E44" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -1935,10 +1935,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E45" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="F45" t="n">
         <v>0</v>
@@ -1969,13 +1969,13 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E46" t="n">
-        <v>1357300</v>
+        <v>1305400</v>
       </c>
       <c r="F46" t="n">
-        <v>27700</v>
+        <v>26600</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -2003,13 +2003,13 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E47" t="n">
-        <v>1343500</v>
+        <v>1292100</v>
       </c>
       <c r="F47" t="n">
-        <v>41500</v>
+        <v>39900</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2037,13 +2037,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E48" t="n">
-        <v>1329600</v>
+        <v>1278800</v>
       </c>
       <c r="F48" t="n">
-        <v>55400</v>
+        <v>53200</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2071,13 +2071,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E49" t="n">
-        <v>1315800</v>
+        <v>1265400</v>
       </c>
       <c r="F49" t="n">
-        <v>69200</v>
+        <v>66600</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2105,10 +2105,10 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E50" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -2139,10 +2139,10 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E51" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -2173,13 +2173,13 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E52" t="n">
-        <v>342100</v>
+        <v>328300</v>
       </c>
       <c r="F52" t="n">
-        <v>6900</v>
+        <v>6700</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -2207,13 +2207,13 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E53" t="n">
-        <v>338600</v>
+        <v>325000</v>
       </c>
       <c r="F53" t="n">
-        <v>10400</v>
+        <v>10000</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -2241,13 +2241,13 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E54" t="n">
-        <v>335100</v>
+        <v>321600</v>
       </c>
       <c r="F54" t="n">
-        <v>13900</v>
+        <v>13400</v>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -2275,13 +2275,13 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E55" t="n">
-        <v>331600</v>
+        <v>318300</v>
       </c>
       <c r="F55" t="n">
-        <v>17400</v>
+        <v>16700</v>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -2309,10 +2309,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E56" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -2343,10 +2343,10 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E57" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -2377,13 +2377,13 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E58" t="n">
-        <v>4623700</v>
+        <v>4449200</v>
       </c>
       <c r="F58" t="n">
-        <v>94300</v>
+        <v>90800</v>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -2411,13 +2411,13 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E59" t="n">
-        <v>4576500</v>
+        <v>4403800</v>
       </c>
       <c r="F59" t="n">
-        <v>141500</v>
+        <v>136200</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -2445,13 +2445,13 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E60" t="n">
-        <v>4529300</v>
+        <v>4358400</v>
       </c>
       <c r="F60" t="n">
-        <v>188700</v>
+        <v>181600</v>
       </c>
       <c r="G60" t="inlineStr">
         <is>
@@ -2479,13 +2479,13 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4718000</v>
+        <v>4540000</v>
       </c>
       <c r="E61" t="n">
-        <v>4482100</v>
+        <v>4313000</v>
       </c>
       <c r="F61" t="n">
-        <v>235900</v>
+        <v>227000</v>
       </c>
       <c r="G61" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E62" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -2547,10 +2547,10 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E63" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -2581,13 +2581,13 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E64" t="n">
-        <v>1357300</v>
+        <v>1305400</v>
       </c>
       <c r="F64" t="n">
-        <v>27700</v>
+        <v>26600</v>
       </c>
       <c r="G64" t="inlineStr">
         <is>
@@ -2615,13 +2615,13 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E65" t="n">
-        <v>1343500</v>
+        <v>1292100</v>
       </c>
       <c r="F65" t="n">
-        <v>41500</v>
+        <v>39900</v>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -2649,13 +2649,13 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E66" t="n">
-        <v>1329600</v>
+        <v>1278800</v>
       </c>
       <c r="F66" t="n">
-        <v>55400</v>
+        <v>53200</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -2683,13 +2683,13 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1385000</v>
+        <v>1332000</v>
       </c>
       <c r="E67" t="n">
-        <v>1315800</v>
+        <v>1265400</v>
       </c>
       <c r="F67" t="n">
-        <v>69200</v>
+        <v>66600</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -2717,10 +2717,10 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E68" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -2751,10 +2751,10 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E69" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
@@ -2785,13 +2785,13 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E70" t="n">
-        <v>342100</v>
+        <v>328300</v>
       </c>
       <c r="F70" t="n">
-        <v>6900</v>
+        <v>6700</v>
       </c>
       <c r="G70" t="inlineStr">
         <is>
@@ -2819,13 +2819,13 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E71" t="n">
-        <v>338600</v>
+        <v>325000</v>
       </c>
       <c r="F71" t="n">
-        <v>10400</v>
+        <v>10000</v>
       </c>
       <c r="G71" t="inlineStr">
         <is>
@@ -2853,13 +2853,13 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E72" t="n">
-        <v>335100</v>
+        <v>321600</v>
       </c>
       <c r="F72" t="n">
-        <v>13900</v>
+        <v>13400</v>
       </c>
       <c r="G72" t="inlineStr">
         <is>
@@ -2887,13 +2887,13 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>349000</v>
+        <v>335000</v>
       </c>
       <c r="E73" t="n">
-        <v>331600</v>
+        <v>318300</v>
       </c>
       <c r="F73" t="n">
-        <v>17400</v>
+        <v>16700</v>
       </c>
       <c r="G73" t="inlineStr">
         <is>

</xml_diff>